<commit_message>
Diagramas unifilar e multifilar dos quadros de distribuição
- Diagramas gerados a partir do dimensionamento: alimentação, disjuntor
  geral, DPS classe II, disjuntores, DR (IDR/DDR), condutores com seções
  e distribuição entre as fases; símbolos IEC 60617 e cores da NBR 5410.
- Unifilar com barramento vertical, marcas de fase/neutro/PE, reserva da
  Tabela 59 e resumo de demanda e equilíbrio; multifilar com barramentos
  A, B, C, N e PE coloridos, polos, toróide do DR e DPS ligados ao PE.
- Seção Quadros: botões unifilar/multifilar, campos de disjuntor geral e
  DPS; documento "Diagramas unifilares e multifilares" em PDF, Word e
  HTML, anexável ao memorial descritivo; DPS na lista de materiais.
- Exportação com figuras de largura total em alta resolução e títulos
  mantidos junto da figura.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E4Px4gvzC9MkKBX1rn21ys
</commit_message>
<xml_diff>
--- a/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
+++ b/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="159">
   <si>
     <t>Lista de materiais</t>
   </si>
@@ -229,6 +229,15 @@
     <t>Dispositivos de proteção</t>
   </si>
   <si>
+    <t>DPS classe II — Uc 175 V, In 20 kA, Imáx 40 kA</t>
+  </si>
+  <si>
+    <t>ABNT NBR IEC 61643-11</t>
+  </si>
+  <si>
+    <t>QM, QD-1</t>
+  </si>
+  <si>
     <t>Disjuntor termomagnético 1P curva C 10 A — 6,0 kA</t>
   </si>
   <si>
@@ -275,9 +284,6 @@
   </si>
   <si>
     <t>DPS classe II — 275 V, In 20 kA, Imáx 40 kA</t>
-  </si>
-  <si>
-    <t>ABNT NBR IEC 61643-11</t>
   </si>
   <si>
     <t>cadastro</t>
@@ -917,7 +923,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1843,7 +1849,7 @@
         <v>15</v>
       </c>
       <c r="G38" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>74</v>
@@ -1860,7 +1866,7 @@
         <v>75</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>14</v>
@@ -1869,10 +1875,10 @@
         <v>15</v>
       </c>
       <c r="G39" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -1883,10 +1889,10 @@
         <v>71</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>14</v>
@@ -1895,10 +1901,10 @@
         <v>15</v>
       </c>
       <c r="G40" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -1909,10 +1915,10 @@
         <v>71</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>14</v>
@@ -1921,10 +1927,10 @@
         <v>15</v>
       </c>
       <c r="G41" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -1935,10 +1941,10 @@
         <v>71</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>14</v>
@@ -1950,7 +1956,7 @@
         <v>1</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1961,10 +1967,10 @@
         <v>71</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>14</v>
@@ -1976,7 +1982,7 @@
         <v>1</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -1987,10 +1993,10 @@
         <v>71</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>14</v>
@@ -1999,10 +2005,10 @@
         <v>15</v>
       </c>
       <c r="G44" s="7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2016,7 +2022,7 @@
         <v>86</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>14</v>
@@ -2025,10 +2031,10 @@
         <v>15</v>
       </c>
       <c r="G45" s="7">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>53</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -2039,11 +2045,11 @@
         <v>71</v>
       </c>
       <c r="C46" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D46" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="D46" s="6" t="s">
-        <v>88</v>
-      </c>
       <c r="E46" s="6" t="s">
         <v>14</v>
       </c>
@@ -2051,10 +2057,10 @@
         <v>15</v>
       </c>
       <c r="G46" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>89</v>
+        <v>53</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2062,25 +2068,25 @@
         <v>42</v>
       </c>
       <c r="B47" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="D47" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G47" s="7">
+        <v>4</v>
+      </c>
+      <c r="H47" s="6" t="s">
         <v>91</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G47" s="7">
-        <v>1</v>
-      </c>
-      <c r="H47" s="6" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2088,13 +2094,13 @@
         <v>43</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C48" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>92</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>14</v>
@@ -2106,7 +2112,7 @@
         <v>1</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2114,13 +2120,13 @@
         <v>44</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>14</v>
@@ -2132,7 +2138,7 @@
         <v>1</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2140,25 +2146,25 @@
         <v>45</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>97</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G50" s="7">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2166,14 +2172,14 @@
         <v>46</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C51" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="D51" s="6" t="s">
-        <v>98</v>
-      </c>
       <c r="E51" s="6" t="s">
         <v>14</v>
       </c>
@@ -2181,7 +2187,7 @@
         <v>25</v>
       </c>
       <c r="G51" s="7">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>101</v>
@@ -2192,13 +2198,13 @@
         <v>47</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>102</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>14</v>
@@ -2207,7 +2213,7 @@
         <v>25</v>
       </c>
       <c r="G52" s="7">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>103</v>
@@ -2218,13 +2224,13 @@
         <v>48</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>104</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>14</v>
@@ -2233,7 +2239,7 @@
         <v>25</v>
       </c>
       <c r="G53" s="7">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="H53" s="6" t="s">
         <v>105</v>
@@ -2244,25 +2250,25 @@
         <v>49</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>106</v>
       </c>
       <c r="D54" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G54" s="7">
+        <v>14</v>
+      </c>
+      <c r="H54" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G54" s="7">
-        <v>14</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -2270,25 +2276,25 @@
         <v>50</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C55" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D55" s="6" t="s">
-        <v>107</v>
-      </c>
       <c r="E55" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G55" s="7">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -2296,13 +2302,13 @@
         <v>51</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>111</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>14</v>
@@ -2311,10 +2317,10 @@
         <v>15</v>
       </c>
       <c r="G56" s="7">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -2322,13 +2328,13 @@
         <v>52</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>113</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>14</v>
@@ -2337,10 +2343,10 @@
         <v>15</v>
       </c>
       <c r="G57" s="7">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -2348,13 +2354,13 @@
         <v>53</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>115</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>14</v>
@@ -2363,10 +2369,10 @@
         <v>15</v>
       </c>
       <c r="G58" s="7">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -2374,13 +2380,13 @@
         <v>54</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>117</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>14</v>
@@ -2389,10 +2395,10 @@
         <v>15</v>
       </c>
       <c r="G59" s="7">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -2400,14 +2406,14 @@
         <v>55</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C60" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D60" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="D60" s="6" t="s">
-        <v>119</v>
-      </c>
       <c r="E60" s="6" t="s">
         <v>14</v>
       </c>
@@ -2415,10 +2421,10 @@
         <v>15</v>
       </c>
       <c r="G60" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
@@ -2426,13 +2432,13 @@
         <v>56</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>120</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>14</v>
@@ -2441,10 +2447,10 @@
         <v>15</v>
       </c>
       <c r="G61" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -2452,14 +2458,14 @@
         <v>57</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C62" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D62" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="D62" s="6" t="s">
-        <v>112</v>
-      </c>
       <c r="E62" s="6" t="s">
         <v>14</v>
       </c>
@@ -2467,10 +2473,10 @@
         <v>15</v>
       </c>
       <c r="G62" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -2478,13 +2484,13 @@
         <v>58</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>123</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>14</v>
@@ -2493,10 +2499,10 @@
         <v>15</v>
       </c>
       <c r="G63" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>125</v>
+        <v>91</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
@@ -2504,13 +2510,13 @@
         <v>59</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C64" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D64" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="D64" s="6" t="s">
-        <v>124</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>14</v>
@@ -2530,13 +2536,13 @@
         <v>60</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>128</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>14</v>
@@ -2545,7 +2551,7 @@
         <v>15</v>
       </c>
       <c r="G65" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H65" s="6" t="s">
         <v>129</v>
@@ -2556,13 +2562,13 @@
         <v>61</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>130</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>14</v>
@@ -2571,7 +2577,7 @@
         <v>15</v>
       </c>
       <c r="G66" s="7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>131</v>
@@ -2582,25 +2588,25 @@
         <v>62</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>132</v>
       </c>
       <c r="D67" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G67" s="7">
+        <v>6</v>
+      </c>
+      <c r="H67" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F67" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G67" s="7">
-        <v>4</v>
-      </c>
-      <c r="H67" s="6" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
@@ -2608,13 +2614,13 @@
         <v>63</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C68" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D68" s="6" t="s">
         <v>135</v>
-      </c>
-      <c r="D68" s="6" t="s">
-        <v>136</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>14</v>
@@ -2626,7 +2632,7 @@
         <v>4</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -2634,7 +2640,7 @@
         <v>64</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>137</v>
@@ -2649,10 +2655,10 @@
         <v>15</v>
       </c>
       <c r="G69" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2660,14 +2666,14 @@
         <v>65</v>
       </c>
       <c r="B70" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C70" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C70" s="6" t="s">
+      <c r="D70" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D70" s="6" t="s">
-        <v>141</v>
-      </c>
       <c r="E70" s="6" t="s">
         <v>14</v>
       </c>
@@ -2675,10 +2681,10 @@
         <v>15</v>
       </c>
       <c r="G70" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -2686,13 +2692,13 @@
         <v>66</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C71" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D71" s="6" t="s">
         <v>143</v>
-      </c>
-      <c r="D71" s="6" t="s">
-        <v>144</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>14</v>
@@ -2704,7 +2710,7 @@
         <v>4</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -2712,13 +2718,13 @@
         <v>67</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>145</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>14</v>
+        <v>146</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>14</v>
@@ -2730,7 +2736,7 @@
         <v>4</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2738,25 +2744,25 @@
         <v>68</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D73" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G73" s="7">
+        <v>4</v>
+      </c>
+      <c r="H73" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="E73" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F73" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G73" s="7">
-        <v>8</v>
-      </c>
-      <c r="H73" s="6" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -2764,25 +2770,25 @@
         <v>69</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D74" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G74" s="7">
+        <v>8</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G74" s="7">
-        <v>3</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2790,13 +2796,13 @@
         <v>70</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>14</v>
@@ -2808,7 +2814,7 @@
         <v>3</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -2816,25 +2822,25 @@
         <v>71</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G76" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>89</v>
+        <v>144</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -2842,14 +2848,14 @@
         <v>72</v>
       </c>
       <c r="B77" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C77" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="C77" s="6" t="s">
+      <c r="D77" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="D77" s="6" t="s">
-        <v>14</v>
-      </c>
       <c r="E77" s="6" t="s">
         <v>14</v>
       </c>
@@ -2857,10 +2863,10 @@
         <v>15</v>
       </c>
       <c r="G77" s="7">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -2868,10 +2874,10 @@
         <v>73</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D78" s="6" t="s">
         <v>14</v>
@@ -2880,13 +2886,13 @@
         <v>14</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>154</v>
+        <v>15</v>
       </c>
       <c r="G78" s="7">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -2894,7 +2900,7 @@
         <v>74</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>155</v>
@@ -2909,14 +2915,40 @@
         <v>156</v>
       </c>
       <c r="G79" s="7">
+        <v>5</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="5">
+        <v>75</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="G80" s="7">
         <v>1</v>
       </c>
-      <c r="H79" s="6" t="s">
-        <v>89</v>
+      <c r="H80" s="6" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H79"/>
+  <autoFilter ref="A5:H80"/>
   <mergeCells count="3">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>

<commit_message>
Módulo SPDA conforme ABNT NBR 5419:2026
- Análise de risco (Parte 2): AD, AM, ND, NM, NL, NI; componentes RA a RZ;
  R1, R3 e frequência de danos F aos sistemas internos; combinações de
  nível de proteção e DPS com o nível mínimo exigido.
- Projeto (Parte 3): NP I a IV, captação em malha ou captores Franklin
  (ângulo equivalente à esfera rolante, sugestão de mastros), descidas,
  anéis, aterramento em anel (arranjo B) com l1 e eletrodos adicionais,
  distância de segurança, materiais e inspeção.
- DPS (Parte 4): Iimp por modo do DPS classe I; quadro de entrada com DPS
  classe I+II nos diagramas e na lista de materiais.
- Seção SPDA no menu Sistemas, memorial PDF/Word/HTML com planta,
  elevação e gráfico de risco, tabela de referência, memorial descritivo
  e exemplo; testes do motor e do navegador.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E4Px4gvzC9MkKBX1rn21ys
</commit_message>
<xml_diff>
--- a/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
+++ b/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="177">
   <si>
     <t>Lista de materiais</t>
   </si>
@@ -19,7 +19,7 @@
     <t>Obra: Residência unifamiliar — exemplo — Proprietário (exemplo)</t>
   </si>
   <si>
-    <t>Sistema: 127/220 V, trifásico, esquema TN-S · Responsável: Nome do responsável técnico — CREA/CFT nº 000000 · R00 · 26/10/2026</t>
+    <t>Sistema: 127/220 V, trifásico, esquema TN-S · Responsável: Nome do responsável técnico — CREA/CFT nº 000000 · R00 · 27/10/2026</t>
   </si>
   <si>
     <t>Item</t>
@@ -229,13 +229,22 @@
     <t>Dispositivos de proteção</t>
   </si>
   <si>
+    <t>DPS classe I+II — Uc 175 V, Iimp 12,5 kA (10/350 µs), In 20 kA</t>
+  </si>
+  <si>
+    <t>ABNT NBR IEC 61643-11; NBR 5419-4</t>
+  </si>
+  <si>
+    <t>QM</t>
+  </si>
+  <si>
     <t>DPS classe II — Uc 175 V, In 20 kA, Imáx 40 kA</t>
   </si>
   <si>
     <t>ABNT NBR IEC 61643-11</t>
   </si>
   <si>
-    <t>QM, QD-1</t>
+    <t>QD-1</t>
   </si>
   <si>
     <t>Disjuntor termomagnético 1P curva C 10 A — 6,0 kA</t>
@@ -298,9 +307,6 @@
     <t>ABNT NBR IEC 61439-3</t>
   </si>
   <si>
-    <t>QD-1</t>
-  </si>
-  <si>
     <t>Barramento de neutro com bornes</t>
   </si>
   <si>
@@ -436,6 +442,57 @@
     <t>ABNT NBR 5123</t>
   </si>
   <si>
+    <t>SPDA — proteção contra descargas atmosféricas</t>
+  </si>
+  <si>
+    <t>Barra chata ou cabo de alumínio 70 mm² — captação (malha e perímetro da cobertura)</t>
+  </si>
+  <si>
+    <t>ABNT NBR 5419-3</t>
+  </si>
+  <si>
+    <t>SPDA</t>
+  </si>
+  <si>
+    <t>Barra chata ou cabo de alumínio 70 mm² — descidas</t>
+  </si>
+  <si>
+    <t>Cabo de cobre nu 50 mm² (7 ou 19 fios) — anel de aterramento a 0,5 m de profundidade e 1,0 m das paredes</t>
+  </si>
+  <si>
+    <t>ABNT NBR 5419-3; NBR 6524</t>
+  </si>
+  <si>
+    <t>Suporte isolador ou fixador para condutor da captação (a cada 1 m)</t>
+  </si>
+  <si>
+    <t>Fixador para condutor de descida (a cada 1 m até 20 m e 0,5 m acima)</t>
+  </si>
+  <si>
+    <t>Conector de cruzamento e emenda da malha de captação</t>
+  </si>
+  <si>
+    <t>Conector de medição (desconexão para ensaio) em cada descida</t>
+  </si>
+  <si>
+    <t>Eletroduto de PVC rígido para proteção mecânica da descida junto ao solo (2,5 m por descida)</t>
+  </si>
+  <si>
+    <t>Caixa de inspeção do aterramento (ligação descida/anel)</t>
+  </si>
+  <si>
+    <t>Conexão por solda exotérmica ou conector de compressão (descida/anel e eletrodos)</t>
+  </si>
+  <si>
+    <t>ABNT NBR 16254</t>
+  </si>
+  <si>
+    <t>Ligação do anel de aterramento ao barramento de equipotencialização principal (BEP)</t>
+  </si>
+  <si>
+    <t>ABNT NBR 5419-3; NBR 5410</t>
+  </si>
+  <si>
     <t>Aterramento e equipotencialização</t>
   </si>
   <si>
@@ -449,9 +506,6 @@
   </si>
   <si>
     <t>Conector cabo–haste (cunha, grampo ou solda exotérmica)</t>
-  </si>
-  <si>
-    <t>ABNT NBR 16254</t>
   </si>
   <si>
     <t>Caixa de inspeção de aterramento com tampa</t>
@@ -923,7 +977,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1849,7 +1903,7 @@
         <v>15</v>
       </c>
       <c r="G38" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>74</v>
@@ -1875,7 +1929,7 @@
         <v>15</v>
       </c>
       <c r="G39" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>77</v>
@@ -1892,7 +1946,7 @@
         <v>78</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>14</v>
@@ -1901,10 +1955,10 @@
         <v>15</v>
       </c>
       <c r="G40" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -1915,10 +1969,10 @@
         <v>71</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>14</v>
@@ -1927,10 +1981,10 @@
         <v>15</v>
       </c>
       <c r="G41" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -1941,10 +1995,10 @@
         <v>71</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>14</v>
@@ -1953,10 +2007,10 @@
         <v>15</v>
       </c>
       <c r="G42" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1967,10 +2021,10 @@
         <v>71</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>14</v>
@@ -1982,7 +2036,7 @@
         <v>1</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -1993,10 +2047,10 @@
         <v>71</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>14</v>
@@ -2008,7 +2062,7 @@
         <v>1</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2019,10 +2073,10 @@
         <v>71</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>14</v>
@@ -2031,10 +2085,10 @@
         <v>15</v>
       </c>
       <c r="G45" s="7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -2048,7 +2102,7 @@
         <v>89</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>14</v>
@@ -2057,10 +2111,10 @@
         <v>15</v>
       </c>
       <c r="G46" s="7">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>53</v>
+        <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2071,11 +2125,11 @@
         <v>71</v>
       </c>
       <c r="C47" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="D47" s="6" t="s">
-        <v>73</v>
-      </c>
       <c r="E47" s="6" t="s">
         <v>14</v>
       </c>
@@ -2083,10 +2137,10 @@
         <v>15</v>
       </c>
       <c r="G47" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>91</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2094,25 +2148,25 @@
         <v>43</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>93</v>
       </c>
       <c r="D48" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" s="7">
+        <v>4</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G48" s="7">
-        <v>1</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2120,13 +2174,13 @@
         <v>44</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>96</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>14</v>
@@ -2138,7 +2192,7 @@
         <v>1</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2146,13 +2200,13 @@
         <v>45</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C50" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>14</v>
@@ -2164,7 +2218,7 @@
         <v>1</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2172,25 +2226,25 @@
         <v>46</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>99</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G51" s="7">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -2198,14 +2252,14 @@
         <v>47</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C52" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D52" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D52" s="6" t="s">
-        <v>100</v>
-      </c>
       <c r="E52" s="6" t="s">
         <v>14</v>
       </c>
@@ -2213,7 +2267,7 @@
         <v>25</v>
       </c>
       <c r="G52" s="7">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>103</v>
@@ -2224,13 +2278,13 @@
         <v>48</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>104</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>14</v>
@@ -2239,7 +2293,7 @@
         <v>25</v>
       </c>
       <c r="G53" s="7">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="H53" s="6" t="s">
         <v>105</v>
@@ -2250,13 +2304,13 @@
         <v>49</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>106</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>14</v>
@@ -2265,7 +2319,7 @@
         <v>25</v>
       </c>
       <c r="G54" s="7">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="H54" s="6" t="s">
         <v>107</v>
@@ -2276,25 +2330,25 @@
         <v>50</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>108</v>
       </c>
       <c r="D55" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G55" s="7">
+        <v>14</v>
+      </c>
+      <c r="H55" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F55" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G55" s="7">
-        <v>14</v>
-      </c>
-      <c r="H55" s="6" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -2302,25 +2356,25 @@
         <v>51</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C56" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D56" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D56" s="6" t="s">
-        <v>109</v>
-      </c>
       <c r="E56" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G56" s="7">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -2328,13 +2382,13 @@
         <v>52</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>113</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>14</v>
@@ -2343,10 +2397,10 @@
         <v>15</v>
       </c>
       <c r="G57" s="7">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -2354,13 +2408,13 @@
         <v>53</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>115</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>14</v>
@@ -2369,10 +2423,10 @@
         <v>15</v>
       </c>
       <c r="G58" s="7">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -2380,13 +2434,13 @@
         <v>54</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>117</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>14</v>
@@ -2395,10 +2449,10 @@
         <v>15</v>
       </c>
       <c r="G59" s="7">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -2406,13 +2460,13 @@
         <v>55</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>119</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>14</v>
@@ -2421,10 +2475,10 @@
         <v>15</v>
       </c>
       <c r="G60" s="7">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
@@ -2432,14 +2486,14 @@
         <v>56</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C61" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D61" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D61" s="6" t="s">
-        <v>121</v>
-      </c>
       <c r="E61" s="6" t="s">
         <v>14</v>
       </c>
@@ -2447,10 +2501,10 @@
         <v>15</v>
       </c>
       <c r="G61" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -2458,13 +2512,13 @@
         <v>57</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>122</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>14</v>
@@ -2473,10 +2527,10 @@
         <v>15</v>
       </c>
       <c r="G62" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -2484,14 +2538,14 @@
         <v>58</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C63" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D63" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="D63" s="6" t="s">
-        <v>114</v>
-      </c>
       <c r="E63" s="6" t="s">
         <v>14</v>
       </c>
@@ -2499,10 +2553,10 @@
         <v>15</v>
       </c>
       <c r="G63" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
@@ -2510,13 +2564,13 @@
         <v>59</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>125</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>14</v>
@@ -2525,10 +2579,10 @@
         <v>15</v>
       </c>
       <c r="G64" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>127</v>
+        <v>94</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
@@ -2536,13 +2590,13 @@
         <v>60</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C65" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D65" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>126</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>14</v>
@@ -2562,13 +2616,13 @@
         <v>61</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>130</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>14</v>
@@ -2577,7 +2631,7 @@
         <v>15</v>
       </c>
       <c r="G66" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>131</v>
@@ -2588,13 +2642,13 @@
         <v>62</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>132</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E67" s="6" t="s">
         <v>14</v>
@@ -2603,7 +2657,7 @@
         <v>15</v>
       </c>
       <c r="G67" s="7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>133</v>
@@ -2614,25 +2668,25 @@
         <v>63</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>134</v>
       </c>
       <c r="D68" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G68" s="7">
+        <v>6</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>135</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F68" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G68" s="7">
-        <v>4</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -2640,13 +2694,13 @@
         <v>64</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C69" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D69" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="D69" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>14</v>
@@ -2658,7 +2712,7 @@
         <v>4</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2666,7 +2720,7 @@
         <v>65</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>139</v>
@@ -2681,10 +2735,10 @@
         <v>15</v>
       </c>
       <c r="G70" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -2692,14 +2746,14 @@
         <v>66</v>
       </c>
       <c r="B71" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C71" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="C71" s="6" t="s">
+      <c r="D71" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="D71" s="6" t="s">
-        <v>143</v>
-      </c>
       <c r="E71" s="6" t="s">
         <v>14</v>
       </c>
@@ -2707,10 +2761,10 @@
         <v>15</v>
       </c>
       <c r="G71" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -2718,25 +2772,25 @@
         <v>67</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C72" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D72" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="D72" s="6" t="s">
+      <c r="E72" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G72" s="7">
+        <v>49</v>
+      </c>
+      <c r="H72" s="6" t="s">
         <v>146</v>
-      </c>
-      <c r="E72" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F72" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G72" s="7">
-        <v>4</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2744,25 +2798,25 @@
         <v>68</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>147</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>14</v>
+        <v>145</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G73" s="7">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -2770,25 +2824,25 @@
         <v>69</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>148</v>
       </c>
       <c r="D74" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G74" s="7">
+        <v>63</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>146</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G74" s="7">
-        <v>8</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2796,25 +2850,25 @@
         <v>70</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D75" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G75" s="7">
+        <v>46</v>
+      </c>
+      <c r="H75" s="6" t="s">
         <v>146</v>
-      </c>
-      <c r="E75" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F75" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G75" s="7">
-        <v>3</v>
-      </c>
-      <c r="H75" s="6" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -2822,25 +2876,25 @@
         <v>71</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G76" s="7">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -2848,13 +2902,13 @@
         <v>72</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>14</v>
@@ -2863,10 +2917,10 @@
         <v>15</v>
       </c>
       <c r="G77" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -2874,13 +2928,13 @@
         <v>73</v>
       </c>
       <c r="B78" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C78" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="C78" s="6" t="s">
-        <v>154</v>
-      </c>
       <c r="D78" s="6" t="s">
-        <v>14</v>
+        <v>145</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>14</v>
@@ -2889,10 +2943,10 @@
         <v>15</v>
       </c>
       <c r="G78" s="7">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -2900,25 +2954,25 @@
         <v>74</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>14</v>
+        <v>102</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>156</v>
+        <v>25</v>
       </c>
       <c r="G79" s="7">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -2926,29 +2980,341 @@
         <v>75</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C80" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G80" s="7">
+        <v>4</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" s="5">
+        <v>76</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D81" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="D80" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E80" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F80" s="5" t="s">
+      <c r="E81" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G81" s="7">
+        <v>4</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" s="5">
+        <v>77</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C82" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="G80" s="7">
+      <c r="D82" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G82" s="7">
         <v>1</v>
       </c>
-      <c r="H80" s="6" t="s">
-        <v>91</v>
+      <c r="H82" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" s="5">
+        <v>78</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G83" s="7">
+        <v>4</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" s="5">
+        <v>79</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E84" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G84" s="7">
+        <v>4</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" s="5">
+        <v>80</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D85" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E85" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G85" s="7">
+        <v>4</v>
+      </c>
+      <c r="H85" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" s="5">
+        <v>81</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E86" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G86" s="7">
+        <v>8</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" s="5">
+        <v>82</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G87" s="7">
+        <v>3</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" s="5">
+        <v>83</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G88" s="7">
+        <v>3</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" s="5">
+        <v>84</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G89" s="7">
+        <v>1</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" s="5">
+        <v>85</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G90" s="7">
+        <v>40</v>
+      </c>
+      <c r="H90" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" s="5">
+        <v>86</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D91" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G91" s="7">
+        <v>5</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="5">
+        <v>87</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D92" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="G92" s="7">
+        <v>1</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H80"/>
+  <autoFilter ref="A5:H92"/>
   <mergeCells count="3">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>

<commit_message>
Motor de DPS por quadro e NG do Anexo F só no motor de cálculo
- Nova seção Instalações › Proteção contra surtos (DPS): classe, ligação
  pelo esquema de aterramento (n+0 ou n+1 com centelhador N–PE), Uc
  (Tabela 49), Up ≤ categoria II (Tabela 31), nível efetivo Up/f,
  In/Imáx pela exposição (faixas usuais de fabricantes), Iimp pelo nível
  do SPDA, condutores de ligação, retaguarda, Isccr, coordenação e
  DPS classe III.
- Memória de cálculo do DPS (PDF, Word, HTML), anexável ao memorial
  descritivo; diagramas com a especificação e o desenho da ligação n+1;
  lista de materiais pelo motor; tabela de referência em Tabelas.
- Memorial do SPDA cita só o município escolhido; a tabela do Anexo F
  (MS) permanece no motor de cálculo.
- Testes do motor e do navegador.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E4Px4gvzC9MkKBX1rn21ys
</commit_message>
<xml_diff>
--- a/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
+++ b/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="178">
   <si>
     <t>Lista de materiais</t>
   </si>
@@ -229,22 +229,25 @@
     <t>Dispositivos de proteção</t>
   </si>
   <si>
-    <t>DPS classe I+II — Uc 175 V, Iimp 12,5 kA (10/350 µs), In 20 kA</t>
-  </si>
-  <si>
-    <t>ABNT NBR IEC 61643-11; NBR 5419-4</t>
+    <t>DPS classe I+II unipolar — Uc 175 V, Iimp 12,5 kA (10/350 µs), In 20 kA, Up ≤ 1,5 kV</t>
+  </si>
+  <si>
+    <t>ABNT NBR IEC 61643-11</t>
   </si>
   <si>
     <t>QM</t>
   </si>
   <si>
-    <t>DPS classe II — Uc 175 V, In 20 kA, Imáx 40 kA</t>
-  </si>
-  <si>
-    <t>ABNT NBR IEC 61643-11</t>
+    <t>Condutor de cobre verde-amarelo 16 mm² para ligação dos DPS</t>
+  </si>
+  <si>
+    <t>DPS classe II unipolar — Uc 175 V, In 20 kA, Imáx 40 kA (8/20 µs), Up ≤ 1,2 kV</t>
   </si>
   <si>
     <t>QD-1</t>
+  </si>
+  <si>
+    <t>Condutor de cobre verde-amarelo 4 mm² para ligação dos DPS</t>
   </si>
   <si>
     <t>Disjuntor termomagnético 1P curva C 10 A — 6,0 kA</t>
@@ -977,7 +980,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1920,19 +1923,19 @@
         <v>75</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>76</v>
+        <v>24</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G39" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -1943,10 +1946,10 @@
         <v>71</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>14</v>
@@ -1955,10 +1958,10 @@
         <v>15</v>
       </c>
       <c r="G40" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -1969,22 +1972,22 @@
         <v>71</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>79</v>
+        <v>24</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G41" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -1995,10 +1998,10 @@
         <v>71</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>14</v>
@@ -2007,10 +2010,10 @@
         <v>15</v>
       </c>
       <c r="G42" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -2021,10 +2024,10 @@
         <v>71</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>14</v>
@@ -2033,10 +2036,10 @@
         <v>15</v>
       </c>
       <c r="G43" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2047,10 +2050,10 @@
         <v>71</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>14</v>
@@ -2059,10 +2062,10 @@
         <v>15</v>
       </c>
       <c r="G44" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2073,10 +2076,10 @@
         <v>71</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>14</v>
@@ -2088,7 +2091,7 @@
         <v>1</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -2099,10 +2102,10 @@
         <v>71</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>14</v>
@@ -2111,10 +2114,10 @@
         <v>15</v>
       </c>
       <c r="G46" s="7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>91</v>
+        <v>53</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2125,10 +2128,10 @@
         <v>71</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>14</v>
@@ -2140,7 +2143,7 @@
         <v>1</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2151,10 +2154,10 @@
         <v>71</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>14</v>
@@ -2163,10 +2166,10 @@
         <v>15</v>
       </c>
       <c r="G48" s="7">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2174,13 +2177,13 @@
         <v>44</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>14</v>
@@ -2192,7 +2195,7 @@
         <v>1</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2200,25 +2203,25 @@
         <v>45</v>
       </c>
       <c r="B50" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G50" s="7">
+        <v>4</v>
+      </c>
+      <c r="H50" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F50" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G50" s="7">
-        <v>1</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2226,13 +2229,13 @@
         <v>46</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>14</v>
@@ -2244,7 +2247,7 @@
         <v>1</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -2252,25 +2255,25 @@
         <v>47</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G52" s="7">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -2278,25 +2281,25 @@
         <v>48</v>
       </c>
       <c r="B53" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C53" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C53" s="6" t="s">
-        <v>104</v>
-      </c>
       <c r="D53" s="6" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G53" s="7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -2304,13 +2307,13 @@
         <v>49</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>14</v>
@@ -2319,10 +2322,10 @@
         <v>25</v>
       </c>
       <c r="G54" s="7">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -2330,13 +2333,13 @@
         <v>50</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>14</v>
@@ -2345,10 +2348,10 @@
         <v>25</v>
       </c>
       <c r="G55" s="7">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -2356,13 +2359,13 @@
         <v>51</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>14</v>
@@ -2371,10 +2374,10 @@
         <v>25</v>
       </c>
       <c r="G56" s="7">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -2382,25 +2385,25 @@
         <v>52</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G57" s="7">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -2408,25 +2411,25 @@
         <v>53</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G58" s="7">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -2434,13 +2437,13 @@
         <v>54</v>
       </c>
       <c r="B59" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C59" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C59" s="6" t="s">
-        <v>117</v>
-      </c>
       <c r="D59" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>14</v>
@@ -2449,10 +2452,10 @@
         <v>15</v>
       </c>
       <c r="G59" s="7">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -2460,13 +2463,13 @@
         <v>55</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>14</v>
@@ -2475,10 +2478,10 @@
         <v>15</v>
       </c>
       <c r="G60" s="7">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
@@ -2486,13 +2489,13 @@
         <v>56</v>
       </c>
       <c r="B61" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C61" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C61" s="6" t="s">
-        <v>121</v>
-      </c>
       <c r="D61" s="6" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>14</v>
@@ -2501,10 +2504,10 @@
         <v>15</v>
       </c>
       <c r="G61" s="7">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -2512,13 +2515,13 @@
         <v>57</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>14</v>
@@ -2527,10 +2530,10 @@
         <v>15</v>
       </c>
       <c r="G62" s="7">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -2538,13 +2541,13 @@
         <v>58</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>14</v>
@@ -2553,10 +2556,10 @@
         <v>15</v>
       </c>
       <c r="G63" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
@@ -2564,13 +2567,13 @@
         <v>59</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>14</v>
@@ -2579,10 +2582,10 @@
         <v>15</v>
       </c>
       <c r="G64" s="7">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
@@ -2590,13 +2593,13 @@
         <v>60</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>14</v>
@@ -2605,10 +2608,10 @@
         <v>15</v>
       </c>
       <c r="G65" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>129</v>
+        <v>95</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
@@ -2616,13 +2619,13 @@
         <v>61</v>
       </c>
       <c r="B66" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C66" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C66" s="6" t="s">
-        <v>130</v>
-      </c>
       <c r="D66" s="6" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>14</v>
@@ -2631,10 +2634,10 @@
         <v>15</v>
       </c>
       <c r="G66" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>131</v>
+        <v>95</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
@@ -2642,13 +2645,13 @@
         <v>62</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E67" s="6" t="s">
         <v>14</v>
@@ -2657,10 +2660,10 @@
         <v>15</v>
       </c>
       <c r="G67" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
@@ -2668,13 +2671,13 @@
         <v>63</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>14</v>
@@ -2683,10 +2686,10 @@
         <v>15</v>
       </c>
       <c r="G68" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -2694,13 +2697,13 @@
         <v>64</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>14</v>
@@ -2709,10 +2712,10 @@
         <v>15</v>
       </c>
       <c r="G69" s="7">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2720,13 +2723,13 @@
         <v>65</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>14</v>
@@ -2735,10 +2738,10 @@
         <v>15</v>
       </c>
       <c r="G70" s="7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -2746,13 +2749,13 @@
         <v>66</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>14</v>
@@ -2761,10 +2764,10 @@
         <v>15</v>
       </c>
       <c r="G71" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -2772,25 +2775,25 @@
         <v>67</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G72" s="7">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2798,25 +2801,25 @@
         <v>68</v>
       </c>
       <c r="B73" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D73" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C73" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="D73" s="6" t="s">
-        <v>145</v>
-      </c>
       <c r="E73" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G73" s="7">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -2824,13 +2827,13 @@
         <v>69</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>14</v>
@@ -2839,10 +2842,10 @@
         <v>25</v>
       </c>
       <c r="G74" s="7">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2850,25 +2853,25 @@
         <v>70</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G75" s="7">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -2876,25 +2879,25 @@
         <v>71</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G76" s="7">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -2902,13 +2905,13 @@
         <v>72</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>14</v>
@@ -2917,10 +2920,10 @@
         <v>15</v>
       </c>
       <c r="G77" s="7">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -2928,13 +2931,13 @@
         <v>73</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>14</v>
@@ -2943,10 +2946,10 @@
         <v>15</v>
       </c>
       <c r="G78" s="7">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -2954,25 +2957,25 @@
         <v>74</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>102</v>
+        <v>146</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G79" s="7">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -2980,13 +2983,13 @@
         <v>75</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>14</v>
@@ -2998,7 +3001,7 @@
         <v>4</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
@@ -3006,25 +3009,25 @@
         <v>76</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>157</v>
+        <v>103</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G81" s="7">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H81" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
@@ -3032,25 +3035,25 @@
         <v>77</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G82" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -3058,13 +3061,13 @@
         <v>78</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>14</v>
@@ -3076,7 +3079,7 @@
         <v>4</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -3084,25 +3087,25 @@
         <v>79</v>
       </c>
       <c r="B84" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D84" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="C84" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="D84" s="6" t="s">
-        <v>157</v>
-      </c>
       <c r="E84" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G84" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
@@ -3110,13 +3113,13 @@
         <v>80</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>14</v>
@@ -3128,7 +3131,7 @@
         <v>4</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -3136,25 +3139,25 @@
         <v>81</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G86" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
@@ -3162,25 +3165,25 @@
         <v>82</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>157</v>
+        <v>14</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G87" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
@@ -3188,13 +3191,13 @@
         <v>83</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>102</v>
+        <v>158</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>14</v>
@@ -3203,10 +3206,10 @@
         <v>25</v>
       </c>
       <c r="G88" s="7">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -3214,25 +3217,25 @@
         <v>84</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F89" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G89" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H89" s="6" t="s">
-        <v>94</v>
+        <v>164</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
@@ -3240,25 +3243,25 @@
         <v>85</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>14</v>
+        <v>103</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F90" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G90" s="7">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>94</v>
+        <v>164</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
@@ -3266,25 +3269,25 @@
         <v>86</v>
       </c>
       <c r="B91" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D91" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="C91" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D91" s="6" t="s">
-        <v>14</v>
-      </c>
       <c r="E91" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>174</v>
+        <v>15</v>
       </c>
       <c r="G91" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
@@ -3292,29 +3295,81 @@
         <v>87</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C92" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D92" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G92" s="7">
+        <v>40</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="5">
+        <v>88</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D93" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="D92" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E92" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F92" s="5" t="s">
+      <c r="G93" s="7">
+        <v>5</v>
+      </c>
+      <c r="H93" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="5">
+        <v>89</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C94" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="G92" s="7">
+      <c r="D94" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="G94" s="7">
         <v>1</v>
       </c>
-      <c r="H92" s="6" t="s">
-        <v>94</v>
+      <c r="H94" s="6" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H92"/>
+  <autoFilter ref="A5:H94"/>
   <mergeCells count="3">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>

<commit_message>
DPS: parâmetros complementares de seleção (TOV, Ifi, lpo, tecnologia, coordenação)
- Sobretensão temporária: UT >= 1,45 x U0 por 5 s; centelhador N-PE no TT
  para 1200 V por 200 ms (IEC 61643-11)
- Tecnologia do DPS classe I: varistor (Up/f = Up + dU) ou centelhador
  (Up/f = max(Up; dU)), com Ifi >= curto-circuito presumido; N-PE Ifi >= 100 A
- Ligação em V (dU desprezível)
- Distância de proteção por oscilação lpo = (Uw - Up/f) / 25 V/m com a lista
  de circuitos terminais mais longos (IEC 62305-4, Anexo D)
- Coordenação entre estágios: 10 m de cabo (IEC 61643-12) ou declaração do
  fabricante; aviso de DR tipo S para DPS a jusante de DR geral
- Memória, tabelas de referência, README e testes atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E4Px4gvzC9MkKBX1rn21ys
</commit_message>
<xml_diff>
--- a/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
+++ b/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="180">
   <si>
     <t>Lista de materiais</t>
   </si>
@@ -229,7 +229,7 @@
     <t>Dispositivos de proteção</t>
   </si>
   <si>
-    <t>DPS classe I+II unipolar — Uc 175 V, Iimp 12,5 kA (10/350 µs), In 20 kA, Up ≤ 1,5 kV</t>
+    <t>DPS classe I+II unipolar (varistor) — Uc 175 V, Iimp 12,5 kA (10/350 µs), In 20 kA, Up ≤ 1,5 kV</t>
   </si>
   <si>
     <t>ABNT NBR IEC 61643-11</t>
@@ -248,6 +248,12 @@
   </si>
   <si>
     <t>Condutor de cobre verde-amarelo 4 mm² para ligação dos DPS</t>
+  </si>
+  <si>
+    <t>DPS classe III junto ao equipamento sensível — Uc 175 V</t>
+  </si>
+  <si>
+    <t>equipamentos sensíveis</t>
   </si>
   <si>
     <t>Disjuntor termomagnético 1P curva C 10 A — 6,0 kA</t>
@@ -980,7 +986,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2001,19 +2007,19 @@
         <v>79</v>
       </c>
       <c r="D42" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42" s="7">
+        <v>2</v>
+      </c>
+      <c r="H42" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G42" s="7">
-        <v>5</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -2024,11 +2030,11 @@
         <v>71</v>
       </c>
       <c r="C43" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D43" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="E43" s="6" t="s">
         <v>14</v>
       </c>
@@ -2036,7 +2042,7 @@
         <v>15</v>
       </c>
       <c r="G43" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>83</v>
@@ -2053,7 +2059,7 @@
         <v>84</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>14</v>
@@ -2062,7 +2068,7 @@
         <v>15</v>
       </c>
       <c r="G44" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>85</v>
@@ -2079,7 +2085,7 @@
         <v>86</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>14</v>
@@ -2088,7 +2094,7 @@
         <v>15</v>
       </c>
       <c r="G45" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>87</v>
@@ -2105,7 +2111,7 @@
         <v>88</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>14</v>
@@ -2117,7 +2123,7 @@
         <v>1</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>53</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2128,10 +2134,10 @@
         <v>71</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>14</v>
@@ -2143,7 +2149,7 @@
         <v>1</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2154,10 +2160,10 @@
         <v>71</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>14</v>
@@ -2166,10 +2172,10 @@
         <v>15</v>
       </c>
       <c r="G48" s="7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2180,11 +2186,11 @@
         <v>71</v>
       </c>
       <c r="C49" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="D49" s="6" t="s">
-        <v>91</v>
-      </c>
       <c r="E49" s="6" t="s">
         <v>14</v>
       </c>
@@ -2192,10 +2198,10 @@
         <v>15</v>
       </c>
       <c r="G49" s="7">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>53</v>
+        <v>94</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2206,10 +2212,10 @@
         <v>71</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>14</v>
@@ -2218,10 +2224,10 @@
         <v>15</v>
       </c>
       <c r="G50" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>95</v>
+        <v>53</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2229,25 +2235,25 @@
         <v>46</v>
       </c>
       <c r="B51" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C51" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="D51" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G51" s="7">
+        <v>4</v>
+      </c>
+      <c r="H51" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F51" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G51" s="7">
-        <v>1</v>
-      </c>
-      <c r="H51" s="6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -2255,13 +2261,13 @@
         <v>47</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>99</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>14</v>
@@ -2273,7 +2279,7 @@
         <v>1</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -2281,13 +2287,13 @@
         <v>48</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C53" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D53" s="6" t="s">
         <v>100</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>14</v>
@@ -2299,7 +2305,7 @@
         <v>1</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -2307,25 +2313,25 @@
         <v>49</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>102</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G54" s="7">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -2333,14 +2339,14 @@
         <v>50</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C55" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D55" s="6" t="s">
-        <v>103</v>
-      </c>
       <c r="E55" s="6" t="s">
         <v>14</v>
       </c>
@@ -2348,7 +2354,7 @@
         <v>25</v>
       </c>
       <c r="G55" s="7">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="H55" s="6" t="s">
         <v>106</v>
@@ -2359,13 +2365,13 @@
         <v>51</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>107</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>14</v>
@@ -2374,7 +2380,7 @@
         <v>25</v>
       </c>
       <c r="G56" s="7">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="H56" s="6" t="s">
         <v>108</v>
@@ -2385,13 +2391,13 @@
         <v>52</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>109</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>14</v>
@@ -2400,7 +2406,7 @@
         <v>25</v>
       </c>
       <c r="G57" s="7">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="H57" s="6" t="s">
         <v>110</v>
@@ -2411,25 +2417,25 @@
         <v>53</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>111</v>
       </c>
       <c r="D58" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G58" s="7">
+        <v>14</v>
+      </c>
+      <c r="H58" s="6" t="s">
         <v>112</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F58" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G58" s="7">
-        <v>14</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -2437,25 +2443,25 @@
         <v>54</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C59" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D59" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D59" s="6" t="s">
-        <v>112</v>
-      </c>
       <c r="E59" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G59" s="7">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -2463,13 +2469,13 @@
         <v>55</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>116</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>14</v>
@@ -2478,10 +2484,10 @@
         <v>15</v>
       </c>
       <c r="G60" s="7">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
@@ -2489,13 +2495,13 @@
         <v>56</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>118</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>14</v>
@@ -2504,10 +2510,10 @@
         <v>15</v>
       </c>
       <c r="G61" s="7">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -2515,13 +2521,13 @@
         <v>57</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>120</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>14</v>
@@ -2530,10 +2536,10 @@
         <v>15</v>
       </c>
       <c r="G62" s="7">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -2541,13 +2547,13 @@
         <v>58</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>122</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>14</v>
@@ -2556,10 +2562,10 @@
         <v>15</v>
       </c>
       <c r="G63" s="7">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
@@ -2567,14 +2573,14 @@
         <v>59</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C64" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D64" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="D64" s="6" t="s">
-        <v>124</v>
-      </c>
       <c r="E64" s="6" t="s">
         <v>14</v>
       </c>
@@ -2582,10 +2588,10 @@
         <v>15</v>
       </c>
       <c r="G64" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
@@ -2593,13 +2599,13 @@
         <v>60</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>125</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>14</v>
@@ -2608,10 +2614,10 @@
         <v>15</v>
       </c>
       <c r="G65" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
@@ -2619,14 +2625,14 @@
         <v>61</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C66" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D66" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D66" s="6" t="s">
-        <v>117</v>
-      </c>
       <c r="E66" s="6" t="s">
         <v>14</v>
       </c>
@@ -2634,10 +2640,10 @@
         <v>15</v>
       </c>
       <c r="G66" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
@@ -2645,13 +2651,13 @@
         <v>62</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>128</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="E67" s="6" t="s">
         <v>14</v>
@@ -2660,10 +2666,10 @@
         <v>15</v>
       </c>
       <c r="G67" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>130</v>
+        <v>97</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
@@ -2671,13 +2677,13 @@
         <v>63</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C68" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D68" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="D68" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>14</v>
@@ -2697,13 +2703,13 @@
         <v>64</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>133</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>14</v>
@@ -2712,7 +2718,7 @@
         <v>15</v>
       </c>
       <c r="G69" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H69" s="6" t="s">
         <v>134</v>
@@ -2723,13 +2729,13 @@
         <v>65</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>135</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>14</v>
@@ -2738,7 +2744,7 @@
         <v>15</v>
       </c>
       <c r="G70" s="7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>136</v>
@@ -2749,25 +2755,25 @@
         <v>66</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>137</v>
       </c>
       <c r="D71" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G71" s="7">
+        <v>6</v>
+      </c>
+      <c r="H71" s="6" t="s">
         <v>138</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F71" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G71" s="7">
-        <v>4</v>
-      </c>
-      <c r="H71" s="6" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -2775,13 +2781,13 @@
         <v>67</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C72" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D72" s="6" t="s">
         <v>140</v>
-      </c>
-      <c r="D72" s="6" t="s">
-        <v>141</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>14</v>
@@ -2793,7 +2799,7 @@
         <v>4</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2801,7 +2807,7 @@
         <v>68</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>142</v>
@@ -2816,10 +2822,10 @@
         <v>15</v>
       </c>
       <c r="G73" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -2827,25 +2833,25 @@
         <v>69</v>
       </c>
       <c r="B74" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C74" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="C74" s="6" t="s">
+      <c r="D74" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="D74" s="6" t="s">
-        <v>146</v>
-      </c>
       <c r="E74" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G74" s="7">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2853,14 +2859,14 @@
         <v>70</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C75" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D75" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="D75" s="6" t="s">
-        <v>146</v>
-      </c>
       <c r="E75" s="6" t="s">
         <v>14</v>
       </c>
@@ -2868,10 +2874,10 @@
         <v>25</v>
       </c>
       <c r="G75" s="7">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -2879,25 +2885,25 @@
         <v>71</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C76" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G76" s="7">
+        <v>28</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>149</v>
-      </c>
-      <c r="D76" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="E76" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F76" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G76" s="7">
-        <v>63</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -2905,25 +2911,25 @@
         <v>72</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>151</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G77" s="7">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -2931,13 +2937,13 @@
         <v>73</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>14</v>
@@ -2946,10 +2952,10 @@
         <v>15</v>
       </c>
       <c r="G78" s="7">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -2957,13 +2963,13 @@
         <v>74</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>14</v>
@@ -2972,10 +2978,10 @@
         <v>15</v>
       </c>
       <c r="G79" s="7">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -2983,13 +2989,13 @@
         <v>75</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>14</v>
@@ -3001,7 +3007,7 @@
         <v>4</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
@@ -3009,25 +3015,25 @@
         <v>76</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>103</v>
+        <v>148</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G81" s="7">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H81" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
@@ -3035,25 +3041,25 @@
         <v>77</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>146</v>
+        <v>105</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G82" s="7">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -3061,13 +3067,13 @@
         <v>78</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>14</v>
@@ -3079,7 +3085,7 @@
         <v>4</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -3087,7 +3093,7 @@
         <v>79</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C84" s="6" t="s">
         <v>159</v>
@@ -3099,13 +3105,13 @@
         <v>14</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G84" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
@@ -3113,25 +3119,25 @@
         <v>80</v>
       </c>
       <c r="B85" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C85" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="C85" s="6" t="s">
+      <c r="D85" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="D85" s="6" t="s">
-        <v>163</v>
-      </c>
       <c r="E85" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G85" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -3139,13 +3145,13 @@
         <v>81</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C86" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D86" s="6" t="s">
         <v>165</v>
-      </c>
-      <c r="D86" s="6" t="s">
-        <v>158</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>14</v>
@@ -3157,7 +3163,7 @@
         <v>4</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
@@ -3165,13 +3171,13 @@
         <v>82</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>14</v>
@@ -3183,7 +3189,7 @@
         <v>4</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
@@ -3191,25 +3197,25 @@
         <v>83</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>158</v>
+        <v>14</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F88" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G88" s="7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -3217,13 +3223,13 @@
         <v>84</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>14</v>
@@ -3232,10 +3238,10 @@
         <v>25</v>
       </c>
       <c r="G89" s="7">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H89" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
@@ -3243,13 +3249,13 @@
         <v>85</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>103</v>
+        <v>160</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>14</v>
@@ -3261,7 +3267,7 @@
         <v>3</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
@@ -3269,25 +3275,25 @@
         <v>86</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>171</v>
+        <v>105</v>
       </c>
       <c r="E91" s="6" t="s">
         <v>14</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G91" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>95</v>
+        <v>166</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
@@ -3295,14 +3301,14 @@
         <v>87</v>
       </c>
       <c r="B92" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C92" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="C92" s="6" t="s">
+      <c r="D92" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D92" s="6" t="s">
-        <v>14</v>
-      </c>
       <c r="E92" s="6" t="s">
         <v>14</v>
       </c>
@@ -3310,10 +3316,10 @@
         <v>15</v>
       </c>
       <c r="G92" s="7">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
@@ -3321,10 +3327,10 @@
         <v>88</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D93" s="6" t="s">
         <v>14</v>
@@ -3333,13 +3339,13 @@
         <v>14</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>175</v>
+        <v>15</v>
       </c>
       <c r="G93" s="7">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
@@ -3347,7 +3353,7 @@
         <v>89</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C94" s="6" t="s">
         <v>176</v>
@@ -3362,14 +3368,40 @@
         <v>177</v>
       </c>
       <c r="G94" s="7">
+        <v>5</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="5">
+        <v>90</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G95" s="7">
         <v>1</v>
       </c>
-      <c r="H94" s="6" t="s">
-        <v>95</v>
+      <c r="H95" s="6" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H94"/>
+  <autoFilter ref="A5:H95"/>
   <mergeCells count="3">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>

<commit_message>
DPS: métodos de fabricantes (catálogo Siemens 5SD7) e retirada do TOV
- Obrigatoriedade pela NBR 5410 (AQ3 com SPDA; AQ2 com linha aérea e Td > 25)
- Corrente nominal da classe II pelo nível de exposição F = Td x (1,6 + 2 LBT + d)
  (In 5/10/20 kA) ou pelas faixas de exposição dos catálogos
- Seção dos condutores de ligação pela proteção a montante, ligação em série (V)
  ou paralelo (T), com fusível F2 quando exigido
- Distância de proteção: lpo (IEC 62305-4) ou 30 m (prática de fabricante)
- Uc e In do produto; Up fase-PE na ligação n+1; neutro aterrado no BEP
  (TN-C-S na entrada) dispensa o módulo N-PE (Figura 13, esquema 1)
- DR a montante com imunidade >= 3 kA (8/20 us); Ifi N-PE >= 100 A (NBR 5410)
- Retirada a verificação de sobretensão temporária (TOV)
- Memória, tabelas de referência, diagramas, README e testes atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E4Px4gvzC9MkKBX1rn21ys
</commit_message>
<xml_diff>
--- a/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
+++ b/exemplo/lista-de-materiais-residencia-unifamiliar-exemplo-r00.xlsx
@@ -238,7 +238,7 @@
     <t>QM</t>
   </si>
   <si>
-    <t>Condutor de cobre verde-amarelo 16 mm² para ligação dos DPS</t>
+    <t>Condutor de cobre 16 mm² para ligação dos DPS (fases e PE)</t>
   </si>
   <si>
     <t>DPS classe II unipolar — Uc 175 V, In 20 kA, Imáx 40 kA (8/20 µs), Up ≤ 1,2 kV</t>
@@ -247,7 +247,7 @@
     <t>QD-1</t>
   </si>
   <si>
-    <t>Condutor de cobre verde-amarelo 4 mm² para ligação dos DPS</t>
+    <t>Condutor de cobre 10 mm² para ligação dos DPS (fases e PE)</t>
   </si>
   <si>
     <t>DPS classe III junto ao equipamento sensível — Uc 175 V</t>

</xml_diff>